<commit_message>
Upgrade to v10: Support all member fields and provide complete custom template
</commit_message>
<xml_diff>
--- a/public/member_template.xlsx
+++ b/public/member_template.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:K3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -410,7 +410,28 @@
         <v>법명</v>
       </c>
       <c r="D1" t="str">
+        <v>법호</v>
+      </c>
+      <c r="E1" t="str">
+        <v>법계</v>
+      </c>
+      <c r="F1" t="str">
+        <v>신분</v>
+      </c>
+      <c r="G1" t="str">
+        <v>직책</v>
+      </c>
+      <c r="H1" t="str">
         <v>소속사찰</v>
+      </c>
+      <c r="I1" t="str">
+        <v>소속사찰직위</v>
+      </c>
+      <c r="J1" t="str">
+        <v>우편번호</v>
+      </c>
+      <c r="K1" t="str">
+        <v>사찰주소</v>
       </c>
     </row>
     <row r="2">
@@ -421,10 +442,31 @@
         <v>010-0000-0000</v>
       </c>
       <c r="C2" t="str">
-        <v/>
+        <v>심원</v>
       </c>
       <c r="D2" t="str">
-        <v/>
+        <v>정연</v>
+      </c>
+      <c r="E2" t="str">
+        <v>전교</v>
+      </c>
+      <c r="F2" t="str">
+        <v>전법사</v>
+      </c>
+      <c r="G2" t="str">
+        <v>총무부장</v>
+      </c>
+      <c r="H2" t="str">
+        <v>수도사</v>
+      </c>
+      <c r="I2" t="str">
+        <v>주지</v>
+      </c>
+      <c r="J2" t="str">
+        <v>12345</v>
+      </c>
+      <c r="K2" t="str">
+        <v>수원시 장안구...</v>
       </c>
     </row>
     <row r="3">
@@ -438,12 +480,33 @@
         <v>아</v>
       </c>
       <c r="D3" t="str">
+        <v>아하</v>
+      </c>
+      <c r="E3" t="str">
+        <v>대장</v>
+      </c>
+      <c r="F3" t="str">
+        <v>비구니</v>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
         <v>수도사</v>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v>수원시 장안구...</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>